<commit_message>
docs(data-model): add dashboard star schema analysis and align with Data Dictionary
</commit_message>
<xml_diff>
--- a/2. Tài liệu phân tích và thiết kế/04. Mô hình dữ liệu/Data_Dictionary_GML.xlsx
+++ b/2. Tài liệu phân tích và thiết kế/04. Mô hình dữ liệu/Data_Dictionary_GML.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Công việc\1. Dự án Gỗ Minh Long\2. Tài liệu phân tích và thiết kế\04. Mô hình dữ liệu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC872D57-C176-4246-BC52-535B1E2920B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C2ADBB3-A600-4C16-959F-B1150873A87A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="7845" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Danh mục " sheetId="21" r:id="rId1"/>
@@ -2095,7 +2095,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2119,43 +2119,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2169,6 +2143,29 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="40% - Accent1" xfId="2" builtinId="31" customBuiltin="1"/>
@@ -2923,20 +2920,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="9" t="s">
         <v>430</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="25" t="s">
         <v>429</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
@@ -3001,7 +2998,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>3</v>
       </c>
@@ -3022,7 +3019,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>4</v>
       </c>
@@ -3087,7 +3084,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>7</v>
       </c>
@@ -3110,7 +3107,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>8</v>
       </c>
@@ -3133,7 +3130,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>9</v>
       </c>
@@ -3236,7 +3233,7 @@
       </c>
       <c r="G17" s="2"/>
     </row>
-    <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>14</v>
       </c>
@@ -3270,7 +3267,7 @@
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
     </row>
-    <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>16</v>
       </c>
@@ -3310,20 +3307,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="26" t="s">
         <v>428</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="26" t="s">
         <v>429</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
@@ -3692,22 +3689,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="25" t="s">
         <v>431</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="25" t="s">
         <v>432</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
@@ -3952,22 +3949,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="26" t="s">
         <v>433</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="26" t="s">
         <v>434</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
@@ -4338,20 +4335,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="26" t="s">
         <v>435</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="26" t="s">
         <v>436</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
@@ -4735,12 +4732,12 @@
       <c r="G8" s="2"/>
     </row>
     <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="F11" s="12" t="s">
+      <c r="F11" s="10" t="s">
         <v>437</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F12" s="12" t="s">
+      <c r="F12" s="10" t="s">
         <v>438</v>
       </c>
     </row>
@@ -4764,20 +4761,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="25" t="s">
         <v>439</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="25" t="s">
         <v>440</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
@@ -4982,22 +4979,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="25" t="s">
         <v>441</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="25" t="s">
         <v>442</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
@@ -5341,22 +5338,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="9" t="s">
         <v>444</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="25" t="s">
         <v>445</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -5766,22 +5763,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="26" t="s">
         <v>446</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="26" t="s">
         <v>447</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
@@ -5869,7 +5866,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>4</v>
       </c>
@@ -5888,7 +5885,7 @@
       </c>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>5</v>
       </c>
@@ -5945,7 +5942,7 @@
       </c>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>8</v>
       </c>
@@ -5966,7 +5963,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>9</v>
       </c>
@@ -5987,7 +5984,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>10</v>
       </c>
@@ -6008,7 +6005,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>11</v>
       </c>
@@ -6029,7 +6026,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>12</v>
       </c>
@@ -6050,7 +6047,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>13</v>
       </c>
@@ -6071,7 +6068,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>14</v>
       </c>
@@ -6109,7 +6106,7 @@
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
     </row>
-    <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>16</v>
       </c>
@@ -6143,7 +6140,7 @@
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
     </row>
-    <row r="22" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>18</v>
       </c>
@@ -6174,1609 +6171,1636 @@
   <dimension ref="A1:B235"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="41.85546875" style="14" customWidth="1"/>
-    <col min="2" max="2" width="41" style="14" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="14"/>
+    <col min="1" max="1" width="41.85546875" style="11" customWidth="1"/>
+    <col min="2" max="2" width="41" style="11" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="11"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="15" t="s">
         <v>452</v>
       </c>
-      <c r="B1" s="26"/>
+      <c r="B1" s="16"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="19"/>
-      <c r="B2" s="20"/>
+      <c r="A2" s="23"/>
+      <c r="B2" s="24"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="17" t="s">
         <v>583</v>
       </c>
-      <c r="B3" s="28"/>
+      <c r="B3" s="18"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="16"/>
-      <c r="B4" s="15"/>
+      <c r="A4" s="13"/>
+      <c r="B4" s="12"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="14" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="4" t="s">
         <v>455</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="4" t="s">
         <v>456</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="4" t="s">
         <v>457</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="4" t="s">
         <v>458</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="4" t="s">
         <v>584</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="21"/>
-      <c r="B11" s="22"/>
+      <c r="A11" s="19"/>
+      <c r="B11" s="20"/>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="23"/>
-      <c r="B12" s="24"/>
+      <c r="A12" s="21"/>
+      <c r="B12" s="22"/>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="27" t="s">
+      <c r="A13" s="17" t="s">
         <v>585</v>
       </c>
-      <c r="B13" s="28"/>
+      <c r="B13" s="18"/>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="16"/>
-      <c r="B14" s="15"/>
+      <c r="A14" s="13"/>
+      <c r="B14" s="12"/>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="17" t="s">
+      <c r="A15" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="B15" s="17" t="s">
+      <c r="B15" s="14" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="18" t="s">
+      <c r="A16" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="B16" s="4" t="s">
         <v>459</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="18" t="s">
+      <c r="A17" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="4" t="s">
         <v>460</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B18" s="18" t="s">
+      <c r="B18" s="4" t="s">
         <v>461</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="21"/>
-      <c r="B19" s="22"/>
+      <c r="A19" s="19"/>
+      <c r="B19" s="20"/>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="23"/>
-      <c r="B20" s="24"/>
+      <c r="A20" s="21"/>
+      <c r="B20" s="22"/>
     </row>
     <row r="21" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="27" t="s">
+      <c r="A21" s="17" t="s">
         <v>586</v>
       </c>
-      <c r="B21" s="28"/>
+      <c r="B21" s="18"/>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="16"/>
-      <c r="B22" s="15"/>
+      <c r="A22" s="13"/>
+      <c r="B22" s="12"/>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="17" t="s">
+      <c r="A23" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="14" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" s="18" t="s">
+      <c r="A24" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B24" s="18" t="s">
+      <c r="B24" s="4" t="s">
         <v>462</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="18" t="s">
+      <c r="A25" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B25" s="18" t="s">
+      <c r="B25" s="4" t="s">
         <v>463</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="18" t="s">
+      <c r="A26" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B26" s="18" t="s">
+      <c r="B26" s="4" t="s">
         <v>464</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="21"/>
-      <c r="B27" s="22"/>
+      <c r="A27" s="19"/>
+      <c r="B27" s="20"/>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="23"/>
-      <c r="B28" s="24"/>
+      <c r="A28" s="21"/>
+      <c r="B28" s="22"/>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="27" t="s">
+      <c r="A29" s="17" t="s">
         <v>587</v>
       </c>
-      <c r="B29" s="28"/>
+      <c r="B29" s="18"/>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="16"/>
-      <c r="B30" s="15"/>
+      <c r="A30" s="13"/>
+      <c r="B30" s="12"/>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="17" t="s">
+      <c r="A31" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="B31" s="17" t="s">
+      <c r="B31" s="14" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A32" s="18" t="s">
+      <c r="A32" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B32" s="18" t="s">
+      <c r="B32" s="4" t="s">
         <v>465</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="18" t="s">
+      <c r="A33" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B33" s="18" t="s">
+      <c r="B33" s="4" t="s">
         <v>466</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A34" s="18" t="s">
+      <c r="A34" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="B34" s="18" t="s">
+      <c r="B34" s="4" t="s">
         <v>467</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" s="18" t="s">
+      <c r="A35" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B35" s="18" t="s">
+      <c r="B35" s="4" t="s">
         <v>468</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" s="21"/>
-      <c r="B36" s="22"/>
+      <c r="A36" s="19"/>
+      <c r="B36" s="20"/>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" s="23"/>
-      <c r="B37" s="24"/>
+      <c r="A37" s="21"/>
+      <c r="B37" s="22"/>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" s="27" t="s">
+      <c r="A38" s="17" t="s">
         <v>588</v>
       </c>
-      <c r="B38" s="28"/>
+      <c r="B38" s="18"/>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" s="16"/>
-      <c r="B39" s="15"/>
+      <c r="A39" s="13"/>
+      <c r="B39" s="12"/>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" s="17" t="s">
+      <c r="A40" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="B40" s="17" t="s">
+      <c r="B40" s="14" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A41" s="18" t="s">
+      <c r="A41" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B41" s="18" t="s">
+      <c r="B41" s="4" t="s">
         <v>469</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="18" t="s">
+      <c r="A42" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B42" s="18" t="s">
+      <c r="B42" s="4" t="s">
         <v>470</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="21"/>
-      <c r="B43" s="22"/>
+      <c r="A43" s="19"/>
+      <c r="B43" s="20"/>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" s="23"/>
-      <c r="B44" s="24"/>
+      <c r="A44" s="21"/>
+      <c r="B44" s="22"/>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" s="27" t="s">
+      <c r="A45" s="17" t="s">
         <v>589</v>
       </c>
-      <c r="B45" s="28"/>
+      <c r="B45" s="18"/>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="16"/>
-      <c r="B46" s="15"/>
+      <c r="A46" s="13"/>
+      <c r="B46" s="12"/>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" s="17" t="s">
+      <c r="A47" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="B47" s="17" t="s">
+      <c r="B47" s="14" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" s="18" t="s">
+      <c r="A48" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="B48" s="18" t="s">
+      <c r="B48" s="4" t="s">
         <v>471</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A49" s="18" t="s">
+      <c r="A49" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B49" s="18" t="s">
+      <c r="B49" s="4" t="s">
         <v>472</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50" s="18" t="s">
+      <c r="A50" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="B50" s="18" t="s">
+      <c r="B50" s="4" t="s">
         <v>473</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A51" s="18" t="s">
+      <c r="A51" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B51" s="18" t="s">
+      <c r="B51" s="4" t="s">
         <v>474</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A52" s="21"/>
-      <c r="B52" s="22"/>
+      <c r="A52" s="19"/>
+      <c r="B52" s="20"/>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A53" s="23"/>
-      <c r="B53" s="24"/>
+      <c r="A53" s="21"/>
+      <c r="B53" s="22"/>
     </row>
     <row r="54" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="27" t="s">
+      <c r="A54" s="17" t="s">
         <v>590</v>
       </c>
-      <c r="B54" s="28"/>
+      <c r="B54" s="18"/>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A55" s="16"/>
-      <c r="B55" s="15"/>
+      <c r="A55" s="13"/>
+      <c r="B55" s="12"/>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A56" s="17" t="s">
+      <c r="A56" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="B56" s="17" t="s">
+      <c r="B56" s="14" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A57" s="18" t="s">
+      <c r="A57" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B57" s="18" t="s">
+      <c r="B57" s="4" t="s">
         <v>475</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A58" s="18" t="s">
+      <c r="A58" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="B58" s="18" t="s">
+      <c r="B58" s="4" t="s">
         <v>591</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A59" s="18" t="s">
+      <c r="A59" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="B59" s="18" t="s">
+      <c r="B59" s="4" t="s">
         <v>476</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A60" s="18" t="s">
+      <c r="A60" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="B60" s="18" t="s">
+      <c r="B60" s="4" t="s">
         <v>477</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A61" s="18" t="s">
+      <c r="A61" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="B61" s="18" t="s">
+      <c r="B61" s="4" t="s">
         <v>478</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A62" s="18" t="s">
+      <c r="A62" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="B62" s="18" t="s">
+      <c r="B62" s="4" t="s">
         <v>479</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A63" s="21"/>
-      <c r="B63" s="22"/>
+      <c r="A63" s="19"/>
+      <c r="B63" s="20"/>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A64" s="23"/>
-      <c r="B64" s="24"/>
+      <c r="A64" s="21"/>
+      <c r="B64" s="22"/>
     </row>
     <row r="65" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="25" t="s">
+      <c r="A65" s="15" t="s">
         <v>480</v>
       </c>
-      <c r="B65" s="26"/>
+      <c r="B65" s="16"/>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A66" s="19"/>
-      <c r="B66" s="20"/>
+      <c r="A66" s="23"/>
+      <c r="B66" s="24"/>
     </row>
     <row r="67" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="27" t="s">
+      <c r="A67" s="17" t="s">
         <v>592</v>
       </c>
-      <c r="B67" s="28"/>
+      <c r="B67" s="18"/>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A68" s="16"/>
-      <c r="B68" s="15"/>
+      <c r="A68" s="13"/>
+      <c r="B68" s="12"/>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A69" s="17" t="s">
+      <c r="A69" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="B69" s="17" t="s">
+      <c r="B69" s="14" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A70" s="18" t="s">
+      <c r="A70" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="B70" s="18" t="s">
+      <c r="B70" s="4" t="s">
         <v>481</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A71" s="18" t="s">
+      <c r="A71" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="B71" s="18" t="s">
+      <c r="B71" s="4" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A72" s="18" t="s">
+      <c r="A72" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="B72" s="18" t="s">
+      <c r="B72" s="4" t="s">
         <v>483</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A73" s="18" t="s">
+      <c r="A73" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="B73" s="18" t="s">
+      <c r="B73" s="4" t="s">
         <v>484</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A74" s="18" t="s">
+      <c r="A74" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B74" s="18" t="s">
+      <c r="B74" s="4" t="s">
         <v>485</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A75" s="18" t="s">
+      <c r="A75" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="B75" s="18" t="s">
+      <c r="B75" s="4" t="s">
         <v>486</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A76" s="18" t="s">
+      <c r="A76" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B76" s="18" t="s">
+      <c r="B76" s="4" t="s">
         <v>487</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A77" s="18" t="s">
+      <c r="A77" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="B77" s="18" t="s">
+      <c r="B77" s="4" t="s">
         <v>488</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A78" s="18" t="s">
+      <c r="A78" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="B78" s="18" t="s">
+      <c r="B78" s="4" t="s">
         <v>489</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A79" s="18" t="s">
+      <c r="A79" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="B79" s="18" t="s">
+      <c r="B79" s="4" t="s">
         <v>490</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A80" s="18" t="s">
+      <c r="A80" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="B80" s="18" t="s">
+      <c r="B80" s="4" t="s">
         <v>491</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A81" s="21"/>
-      <c r="B81" s="22"/>
+      <c r="A81" s="19"/>
+      <c r="B81" s="20"/>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A82" s="23"/>
-      <c r="B82" s="24"/>
+      <c r="A82" s="21"/>
+      <c r="B82" s="22"/>
     </row>
     <row r="83" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="27" t="s">
+      <c r="A83" s="17" t="s">
         <v>593</v>
       </c>
-      <c r="B83" s="28"/>
+      <c r="B83" s="18"/>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A84" s="16"/>
-      <c r="B84" s="15"/>
+      <c r="A84" s="13"/>
+      <c r="B84" s="12"/>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A85" s="17" t="s">
+      <c r="A85" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="B85" s="17" t="s">
+      <c r="B85" s="14" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A86" s="18" t="s">
+      <c r="A86" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="B86" s="18" t="s">
+      <c r="B86" s="4" t="s">
         <v>492</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A87" s="18" t="s">
+      <c r="A87" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="B87" s="18" t="s">
+      <c r="B87" s="4" t="s">
         <v>493</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A88" s="18" t="s">
+      <c r="A88" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="B88" s="18" t="s">
+      <c r="B88" s="4" t="s">
         <v>494</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A89" s="18" t="s">
+      <c r="A89" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="B89" s="18" t="s">
+      <c r="B89" s="4" t="s">
         <v>495</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A90" s="18" t="s">
+      <c r="A90" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B90" s="18" t="s">
+      <c r="B90" s="4" t="s">
         <v>496</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A91" s="18" t="s">
+      <c r="A91" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="B91" s="18" t="s">
+      <c r="B91" s="4" t="s">
         <v>497</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A92" s="18" t="s">
+      <c r="A92" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B92" s="18" t="s">
+      <c r="B92" s="4" t="s">
         <v>498</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A93" s="18" t="s">
+      <c r="A93" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="B93" s="18" t="s">
+      <c r="B93" s="4" t="s">
         <v>499</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A94" s="18" t="s">
+      <c r="A94" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="B94" s="18" t="s">
+      <c r="B94" s="4" t="s">
         <v>500</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A95" s="18" t="s">
+      <c r="A95" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="B95" s="18" t="s">
+      <c r="B95" s="4" t="s">
         <v>501</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A96" s="18" t="s">
+      <c r="A96" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="B96" s="18" t="s">
+      <c r="B96" s="4" t="s">
         <v>502</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A97" s="21"/>
-      <c r="B97" s="22"/>
+      <c r="A97" s="19"/>
+      <c r="B97" s="20"/>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A98" s="23"/>
-      <c r="B98" s="24"/>
+      <c r="A98" s="21"/>
+      <c r="B98" s="22"/>
     </row>
     <row r="99" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A99" s="27" t="s">
+      <c r="A99" s="17" t="s">
         <v>594</v>
       </c>
-      <c r="B99" s="28"/>
+      <c r="B99" s="18"/>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A100" s="16"/>
-      <c r="B100" s="15"/>
+      <c r="A100" s="13"/>
+      <c r="B100" s="12"/>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A101" s="17" t="s">
+      <c r="A101" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="B101" s="17" t="s">
+      <c r="B101" s="14" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A102" s="18" t="s">
+      <c r="A102" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="B102" s="18" t="s">
+      <c r="B102" s="4" t="s">
         <v>503</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A103" s="18" t="s">
+      <c r="A103" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="B103" s="18" t="s">
+      <c r="B103" s="4" t="s">
         <v>504</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A104" s="18" t="s">
+      <c r="A104" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B104" s="18" t="s">
+      <c r="B104" s="4" t="s">
         <v>505</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A105" s="18" t="s">
+      <c r="A105" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="B105" s="18" t="s">
+      <c r="B105" s="4" t="s">
         <v>506</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A106" s="18" t="s">
+      <c r="A106" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="B106" s="18" t="s">
+      <c r="B106" s="4" t="s">
         <v>507</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A107" s="21"/>
-      <c r="B107" s="22"/>
+      <c r="A107" s="19"/>
+      <c r="B107" s="20"/>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A108" s="23"/>
-      <c r="B108" s="24"/>
+      <c r="A108" s="21"/>
+      <c r="B108" s="22"/>
     </row>
     <row r="109" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="27" t="s">
+      <c r="A109" s="17" t="s">
         <v>595</v>
       </c>
-      <c r="B109" s="28"/>
+      <c r="B109" s="18"/>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A110" s="16"/>
-      <c r="B110" s="15"/>
+      <c r="A110" s="13"/>
+      <c r="B110" s="12"/>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A111" s="17" t="s">
+      <c r="A111" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="B111" s="17" t="s">
+      <c r="B111" s="14" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A112" s="18" t="s">
+      <c r="A112" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="B112" s="18" t="s">
+      <c r="B112" s="4" t="s">
         <v>508</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A113" s="18" t="s">
+      <c r="A113" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="B113" s="18" t="s">
+      <c r="B113" s="4" t="s">
         <v>509</v>
       </c>
     </row>
     <row r="114" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A114" s="18" t="s">
+      <c r="A114" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="B114" s="18" t="s">
+      <c r="B114" s="4" t="s">
         <v>510</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A115" s="18" t="s">
+      <c r="A115" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="B115" s="18" t="s">
+      <c r="B115" s="4" t="s">
         <v>511</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A116" s="18" t="s">
+      <c r="A116" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="B116" s="18" t="s">
+      <c r="B116" s="4" t="s">
         <v>512</v>
       </c>
     </row>
     <row r="117" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A117" s="18" t="s">
+      <c r="A117" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B117" s="18" t="s">
+      <c r="B117" s="4" t="s">
         <v>513</v>
       </c>
     </row>
     <row r="118" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A118" s="18" t="s">
+      <c r="A118" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="B118" s="18" t="s">
+      <c r="B118" s="4" t="s">
         <v>581</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A119" s="18" t="s">
+      <c r="A119" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="B119" s="18" t="s">
+      <c r="B119" s="4" t="s">
         <v>582</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A120" s="18" t="s">
+      <c r="A120" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="B120" s="18" t="s">
+      <c r="B120" s="4" t="s">
         <v>514</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A121" s="18" t="s">
+      <c r="A121" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="B121" s="18" t="s">
+      <c r="B121" s="4" t="s">
         <v>515</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A122" s="18" t="s">
+      <c r="A122" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B122" s="18" t="s">
+      <c r="B122" s="4" t="s">
         <v>516</v>
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A123" s="21"/>
-      <c r="B123" s="22"/>
+      <c r="A123" s="19"/>
+      <c r="B123" s="20"/>
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A124" s="23"/>
-      <c r="B124" s="24"/>
+      <c r="A124" s="21"/>
+      <c r="B124" s="22"/>
     </row>
     <row r="125" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A125" s="27" t="s">
+      <c r="A125" s="17" t="s">
         <v>596</v>
       </c>
-      <c r="B125" s="28"/>
+      <c r="B125" s="18"/>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A126" s="16"/>
-      <c r="B126" s="15"/>
+      <c r="A126" s="13"/>
+      <c r="B126" s="12"/>
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A127" s="17" t="s">
+      <c r="A127" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="B127" s="17" t="s">
+      <c r="B127" s="14" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A128" s="18" t="s">
+      <c r="A128" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="B128" s="18" t="s">
+      <c r="B128" s="4" t="s">
         <v>517</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A129" s="18" t="s">
+      <c r="A129" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="B129" s="18" t="s">
+      <c r="B129" s="4" t="s">
         <v>518</v>
       </c>
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A130" s="18" t="s">
+      <c r="A130" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="B130" s="18" t="s">
+      <c r="B130" s="4" t="s">
         <v>519</v>
       </c>
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A131" s="18" t="s">
+      <c r="A131" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="B131" s="18" t="s">
+      <c r="B131" s="4" t="s">
         <v>520</v>
       </c>
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A132" s="18" t="s">
+      <c r="A132" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="B132" s="18" t="s">
+      <c r="B132" s="4" t="s">
         <v>521</v>
       </c>
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A133" s="21"/>
-      <c r="B133" s="22"/>
+      <c r="A133" s="19"/>
+      <c r="B133" s="20"/>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A134" s="23"/>
-      <c r="B134" s="24"/>
+      <c r="A134" s="21"/>
+      <c r="B134" s="22"/>
     </row>
     <row r="135" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A135" s="27" t="s">
+      <c r="A135" s="17" t="s">
         <v>597</v>
       </c>
-      <c r="B135" s="28"/>
+      <c r="B135" s="18"/>
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A136" s="16"/>
-      <c r="B136" s="15"/>
+      <c r="A136" s="13"/>
+      <c r="B136" s="12"/>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A137" s="17" t="s">
+      <c r="A137" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="B137" s="17" t="s">
+      <c r="B137" s="14" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="138" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A138" s="18" t="s">
+      <c r="A138" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="B138" s="18" t="s">
+      <c r="B138" s="4" t="s">
         <v>522</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A139" s="18" t="s">
+      <c r="A139" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="B139" s="18" t="s">
+      <c r="B139" s="4" t="s">
         <v>523</v>
       </c>
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A140" s="18" t="s">
+      <c r="A140" s="4" t="s">
         <v>210</v>
       </c>
-      <c r="B140" s="18" t="s">
+      <c r="B140" s="4" t="s">
         <v>524</v>
       </c>
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A141" s="21"/>
-      <c r="B141" s="22"/>
+      <c r="A141" s="19"/>
+      <c r="B141" s="20"/>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A142" s="23"/>
-      <c r="B142" s="24"/>
+      <c r="A142" s="21"/>
+      <c r="B142" s="22"/>
     </row>
     <row r="143" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A143" s="27" t="s">
+      <c r="A143" s="17" t="s">
         <v>598</v>
       </c>
-      <c r="B143" s="28"/>
+      <c r="B143" s="18"/>
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A144" s="16"/>
-      <c r="B144" s="15"/>
+      <c r="A144" s="13"/>
+      <c r="B144" s="12"/>
     </row>
     <row r="145" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A145" s="17" t="s">
+      <c r="A145" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="B145" s="17" t="s">
+      <c r="B145" s="14" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A146" s="18" t="s">
+      <c r="A146" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="B146" s="18" t="s">
+      <c r="B146" s="4" t="s">
         <v>525</v>
       </c>
     </row>
     <row r="147" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A147" s="18" t="s">
+      <c r="A147" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="B147" s="18" t="s">
+      <c r="B147" s="4" t="s">
         <v>526</v>
       </c>
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A148" s="18" t="s">
+      <c r="A148" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="B148" s="18" t="s">
+      <c r="B148" s="4" t="s">
         <v>527</v>
       </c>
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A149" s="18" t="s">
+      <c r="A149" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="B149" s="18" t="s">
+      <c r="B149" s="4" t="s">
         <v>528</v>
       </c>
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A150" s="21"/>
-      <c r="B150" s="22"/>
+      <c r="A150" s="19"/>
+      <c r="B150" s="20"/>
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A151" s="23"/>
-      <c r="B151" s="24"/>
+      <c r="A151" s="21"/>
+      <c r="B151" s="22"/>
     </row>
     <row r="152" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A152" s="27" t="s">
+      <c r="A152" s="17" t="s">
         <v>599</v>
       </c>
-      <c r="B152" s="28"/>
+      <c r="B152" s="18"/>
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A153" s="16"/>
-      <c r="B153" s="15"/>
+      <c r="A153" s="13"/>
+      <c r="B153" s="12"/>
     </row>
     <row r="154" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A154" s="17" t="s">
+      <c r="A154" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="B154" s="17" t="s">
+      <c r="B154" s="14" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="155" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A155" s="18" t="s">
+      <c r="A155" s="4" t="s">
         <v>239</v>
       </c>
-      <c r="B155" s="18" t="s">
+      <c r="B155" s="4" t="s">
         <v>529</v>
       </c>
     </row>
     <row r="156" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A156" s="18" t="s">
+      <c r="A156" s="4" t="s">
         <v>242</v>
       </c>
-      <c r="B156" s="18" t="s">
+      <c r="B156" s="4" t="s">
         <v>530</v>
       </c>
     </row>
     <row r="157" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A157" s="18" t="s">
+      <c r="A157" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="B157" s="18" t="s">
+      <c r="B157" s="4" t="s">
         <v>531</v>
       </c>
     </row>
     <row r="158" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A158" s="18" t="s">
+      <c r="A158" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B158" s="18" t="s">
+      <c r="B158" s="4" t="s">
         <v>532</v>
       </c>
     </row>
     <row r="159" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A159" s="18" t="s">
+      <c r="A159" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="B159" s="18" t="s">
+      <c r="B159" s="4" t="s">
         <v>533</v>
       </c>
     </row>
     <row r="160" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A160" s="18" t="s">
+      <c r="A160" s="4" t="s">
         <v>230</v>
       </c>
-      <c r="B160" s="18" t="s">
+      <c r="B160" s="4" t="s">
         <v>534</v>
       </c>
     </row>
     <row r="161" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A161" s="18" t="s">
+      <c r="A161" s="4" t="s">
         <v>227</v>
       </c>
-      <c r="B161" s="18" t="s">
+      <c r="B161" s="4" t="s">
         <v>535</v>
       </c>
     </row>
     <row r="162" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A162" s="18" t="s">
+      <c r="A162" s="4" t="s">
         <v>233</v>
       </c>
-      <c r="B162" s="18" t="s">
+      <c r="B162" s="4" t="s">
         <v>536</v>
       </c>
     </row>
     <row r="163" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A163" s="18" t="s">
+      <c r="A163" s="4" t="s">
         <v>236</v>
       </c>
-      <c r="B163" s="18" t="s">
+      <c r="B163" s="4" t="s">
         <v>537</v>
       </c>
     </row>
     <row r="164" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A164" s="21"/>
-      <c r="B164" s="22"/>
+      <c r="A164" s="19"/>
+      <c r="B164" s="20"/>
     </row>
     <row r="165" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A165" s="23"/>
-      <c r="B165" s="24"/>
+      <c r="A165" s="21"/>
+      <c r="B165" s="22"/>
     </row>
     <row r="166" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A166" s="27" t="s">
+      <c r="A166" s="17" t="s">
         <v>600</v>
       </c>
-      <c r="B166" s="28"/>
+      <c r="B166" s="18"/>
     </row>
     <row r="167" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A167" s="16"/>
-      <c r="B167" s="15"/>
+      <c r="A167" s="13"/>
+      <c r="B167" s="12"/>
     </row>
     <row r="168" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A168" s="17" t="s">
+      <c r="A168" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="B168" s="17" t="s">
+      <c r="B168" s="14" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="169" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A169" s="18" t="s">
+      <c r="A169" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="B169" s="18" t="s">
+      <c r="B169" s="4" t="s">
         <v>538</v>
       </c>
     </row>
     <row r="170" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A170" s="18" t="s">
+      <c r="A170" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B170" s="18" t="s">
+      <c r="B170" s="4" t="s">
         <v>539</v>
       </c>
     </row>
     <row r="171" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A171" s="18" t="s">
+      <c r="A171" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="B171" s="18" t="s">
+      <c r="B171" s="4" t="s">
         <v>540</v>
       </c>
     </row>
     <row r="172" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A172" s="18" t="s">
+      <c r="A172" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="B172" s="18" t="s">
+      <c r="B172" s="4" t="s">
         <v>541</v>
       </c>
     </row>
     <row r="173" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A173" s="18" t="s">
+      <c r="A173" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="B173" s="18" t="s">
+      <c r="B173" s="4" t="s">
         <v>542</v>
       </c>
     </row>
     <row r="174" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A174" s="18" t="s">
+      <c r="A174" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="B174" s="18" t="s">
+      <c r="B174" s="4" t="s">
         <v>543</v>
       </c>
     </row>
     <row r="175" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A175" s="18" t="s">
+      <c r="A175" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="B175" s="18" t="s">
+      <c r="B175" s="4" t="s">
         <v>544</v>
       </c>
     </row>
     <row r="176" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A176" s="18" t="s">
+      <c r="A176" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="B176" s="18" t="s">
+      <c r="B176" s="4" t="s">
         <v>545</v>
       </c>
     </row>
     <row r="177" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A177" s="18" t="s">
+      <c r="A177" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="B177" s="18" t="s">
+      <c r="B177" s="4" t="s">
         <v>546</v>
       </c>
     </row>
     <row r="178" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A178" s="18" t="s">
+      <c r="A178" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="B178" s="18" t="s">
+      <c r="B178" s="4" t="s">
         <v>547</v>
       </c>
     </row>
     <row r="179" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A179" s="18" t="s">
+      <c r="A179" s="4" t="s">
         <v>264</v>
       </c>
-      <c r="B179" s="18" t="s">
+      <c r="B179" s="4" t="s">
         <v>548</v>
       </c>
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A180" s="18" t="s">
+      <c r="A180" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="B180" s="18" t="s">
+      <c r="B180" s="4" t="s">
         <v>499</v>
       </c>
     </row>
     <row r="181" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A181" s="18" t="s">
+      <c r="A181" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="B181" s="18" t="s">
+      <c r="B181" s="4" t="s">
         <v>549</v>
       </c>
     </row>
     <row r="182" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A182" s="21"/>
-      <c r="B182" s="22"/>
+      <c r="A182" s="19"/>
+      <c r="B182" s="20"/>
     </row>
     <row r="183" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A183" s="23"/>
-      <c r="B183" s="24"/>
+      <c r="A183" s="21"/>
+      <c r="B183" s="22"/>
     </row>
     <row r="184" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A184" s="27" t="s">
+      <c r="A184" s="17" t="s">
         <v>601</v>
       </c>
-      <c r="B184" s="28"/>
+      <c r="B184" s="18"/>
     </row>
     <row r="185" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A185" s="16"/>
-      <c r="B185" s="15"/>
+      <c r="A185" s="13"/>
+      <c r="B185" s="12"/>
     </row>
     <row r="186" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A186" s="17" t="s">
+      <c r="A186" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="B186" s="17" t="s">
+      <c r="B186" s="14" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="187" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A187" s="18" t="s">
+      <c r="A187" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="B187" s="18" t="s">
+      <c r="B187" s="4" t="s">
         <v>550</v>
       </c>
     </row>
     <row r="188" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A188" s="18" t="s">
+      <c r="A188" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B188" s="18" t="s">
+      <c r="B188" s="4" t="s">
         <v>551</v>
       </c>
     </row>
     <row r="189" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A189" s="18" t="s">
+      <c r="A189" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="B189" s="18" t="s">
+      <c r="B189" s="4" t="s">
         <v>552</v>
       </c>
     </row>
     <row r="190" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A190" s="18" t="s">
+      <c r="A190" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="B190" s="18" t="s">
+      <c r="B190" s="4" t="s">
         <v>553</v>
       </c>
     </row>
     <row r="191" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A191" s="18" t="s">
+      <c r="A191" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="B191" s="18" t="s">
+      <c r="B191" s="4" t="s">
         <v>495</v>
       </c>
     </row>
     <row r="192" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A192" s="18" t="s">
+      <c r="A192" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="B192" s="18" t="s">
+      <c r="B192" s="4" t="s">
         <v>554</v>
       </c>
     </row>
     <row r="193" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A193" s="18" t="s">
+      <c r="A193" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="B193" s="18" t="s">
+      <c r="B193" s="4" t="s">
         <v>555</v>
       </c>
     </row>
     <row r="194" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A194" s="18" t="s">
+      <c r="A194" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="B194" s="18" t="s">
+      <c r="B194" s="4" t="s">
         <v>556</v>
       </c>
     </row>
     <row r="195" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A195" s="18" t="s">
+      <c r="A195" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="B195" s="18" t="s">
+      <c r="B195" s="4" t="s">
         <v>557</v>
       </c>
     </row>
     <row r="196" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A196" s="18" t="s">
+      <c r="A196" s="4" t="s">
         <v>264</v>
       </c>
-      <c r="B196" s="18" t="s">
+      <c r="B196" s="4" t="s">
         <v>558</v>
       </c>
     </row>
     <row r="197" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A197" s="18" t="s">
+      <c r="A197" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="B197" s="18" t="s">
+      <c r="B197" s="4" t="s">
         <v>559</v>
       </c>
     </row>
     <row r="198" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A198" s="18" t="s">
+      <c r="A198" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="B198" s="18" t="s">
+      <c r="B198" s="4" t="s">
         <v>499</v>
       </c>
     </row>
     <row r="199" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A199" s="18" t="s">
+      <c r="A199" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="B199" s="18" t="s">
+      <c r="B199" s="4" t="s">
         <v>549</v>
       </c>
     </row>
     <row r="200" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A200" s="21"/>
-      <c r="B200" s="22"/>
+      <c r="A200" s="19"/>
+      <c r="B200" s="20"/>
     </row>
     <row r="201" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A201" s="23"/>
-      <c r="B201" s="24"/>
+      <c r="A201" s="21"/>
+      <c r="B201" s="22"/>
     </row>
     <row r="202" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A202" s="27" t="s">
+      <c r="A202" s="17" t="s">
         <v>602</v>
       </c>
-      <c r="B202" s="28"/>
+      <c r="B202" s="18"/>
     </row>
     <row r="203" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A203" s="16"/>
-      <c r="B203" s="15"/>
+      <c r="A203" s="13"/>
+      <c r="B203" s="12"/>
     </row>
     <row r="204" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A204" s="17" t="s">
+      <c r="A204" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="B204" s="17" t="s">
+      <c r="B204" s="14" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="205" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A205" s="18" t="s">
+      <c r="A205" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B205" s="18" t="s">
+      <c r="B205" s="4" t="s">
         <v>560</v>
       </c>
     </row>
     <row r="206" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A206" s="18" t="s">
+      <c r="A206" s="4" t="s">
         <v>276</v>
       </c>
-      <c r="B206" s="18" t="s">
+      <c r="B206" s="4" t="s">
         <v>561</v>
       </c>
     </row>
     <row r="207" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A207" s="18" t="s">
+      <c r="A207" s="4" t="s">
         <v>284</v>
       </c>
-      <c r="B207" s="18" t="s">
+      <c r="B207" s="4" t="s">
         <v>562</v>
       </c>
     </row>
     <row r="208" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A208" s="18" t="s">
+      <c r="A208" s="4" t="s">
         <v>279</v>
       </c>
-      <c r="B208" s="18" t="s">
+      <c r="B208" s="4" t="s">
         <v>563</v>
       </c>
     </row>
     <row r="209" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A209" s="18" t="s">
+      <c r="A209" s="4" t="s">
         <v>282</v>
       </c>
-      <c r="B209" s="18" t="s">
+      <c r="B209" s="4" t="s">
         <v>564</v>
       </c>
     </row>
     <row r="210" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A210" s="18" t="s">
+      <c r="A210" s="4" t="s">
         <v>286</v>
       </c>
-      <c r="B210" s="18" t="s">
+      <c r="B210" s="4" t="s">
         <v>565</v>
       </c>
     </row>
     <row r="211" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A211" s="18" t="s">
+      <c r="A211" s="4" t="s">
         <v>227</v>
       </c>
-      <c r="B211" s="18" t="s">
+      <c r="B211" s="4" t="s">
         <v>566</v>
       </c>
     </row>
     <row r="212" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A212" s="21"/>
-      <c r="B212" s="22"/>
+      <c r="A212" s="19"/>
+      <c r="B212" s="20"/>
     </row>
     <row r="213" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A213" s="23"/>
-      <c r="B213" s="24"/>
+      <c r="A213" s="21"/>
+      <c r="B213" s="22"/>
     </row>
     <row r="214" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A214" s="27" t="s">
+      <c r="A214" s="17" t="s">
         <v>603</v>
       </c>
-      <c r="B214" s="28"/>
+      <c r="B214" s="18"/>
     </row>
     <row r="215" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A215" s="16"/>
-      <c r="B215" s="15"/>
+      <c r="A215" s="13"/>
+      <c r="B215" s="12"/>
     </row>
     <row r="216" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A216" s="17" t="s">
+      <c r="A216" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="B216" s="17" t="s">
+      <c r="B216" s="14" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="217" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A217" s="18" t="s">
+      <c r="A217" s="4" t="s">
         <v>304</v>
       </c>
-      <c r="B217" s="18" t="s">
+      <c r="B217" s="4" t="s">
         <v>567</v>
       </c>
     </row>
     <row r="218" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A218" s="18" t="s">
+      <c r="A218" s="4" t="s">
         <v>242</v>
       </c>
-      <c r="B218" s="18" t="s">
+      <c r="B218" s="4" t="s">
         <v>568</v>
       </c>
     </row>
     <row r="219" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A219" s="18" t="s">
+      <c r="A219" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B219" s="18" t="s">
+      <c r="B219" s="4" t="s">
         <v>569</v>
       </c>
     </row>
     <row r="220" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A220" s="18" t="s">
+      <c r="A220" s="4" t="s">
         <v>293</v>
       </c>
-      <c r="B220" s="18" t="s">
+      <c r="B220" s="4" t="s">
         <v>570</v>
       </c>
     </row>
     <row r="221" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A221" s="18" t="s">
+      <c r="A221" s="4" t="s">
         <v>296</v>
       </c>
-      <c r="B221" s="18" t="s">
+      <c r="B221" s="4" t="s">
         <v>571</v>
       </c>
     </row>
     <row r="222" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A222" s="18" t="s">
+      <c r="A222" s="4" t="s">
         <v>299</v>
       </c>
-      <c r="B222" s="18" t="s">
+      <c r="B222" s="4" t="s">
         <v>572</v>
       </c>
     </row>
     <row r="223" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A223" s="18" t="s">
+      <c r="A223" s="4" t="s">
         <v>308</v>
       </c>
-      <c r="B223" s="18" t="s">
+      <c r="B223" s="4" t="s">
         <v>573</v>
       </c>
     </row>
     <row r="224" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A224" s="18" t="s">
+      <c r="A224" s="4" t="s">
         <v>227</v>
       </c>
-      <c r="B224" s="18" t="s">
+      <c r="B224" s="4" t="s">
         <v>574</v>
       </c>
     </row>
     <row r="225" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A225" s="21"/>
-      <c r="B225" s="22"/>
+      <c r="A225" s="19"/>
+      <c r="B225" s="20"/>
     </row>
     <row r="226" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A226" s="23"/>
-      <c r="B226" s="24"/>
+      <c r="A226" s="21"/>
+      <c r="B226" s="22"/>
     </row>
     <row r="227" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A227" s="27" t="s">
+      <c r="A227" s="17" t="s">
         <v>604</v>
       </c>
-      <c r="B227" s="28"/>
+      <c r="B227" s="18"/>
     </row>
     <row r="228" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A228" s="16"/>
-      <c r="B228" s="15"/>
+      <c r="A228" s="13"/>
+      <c r="B228" s="12"/>
     </row>
     <row r="229" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A229" s="17" t="s">
+      <c r="A229" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="B229" s="17" t="s">
+      <c r="B229" s="14" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="230" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A230" s="18" t="s">
+      <c r="A230" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B230" s="18" t="s">
+      <c r="B230" s="4" t="s">
         <v>575</v>
       </c>
     </row>
     <row r="231" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A231" s="18" t="s">
+      <c r="A231" s="4" t="s">
         <v>312</v>
       </c>
-      <c r="B231" s="18" t="s">
+      <c r="B231" s="4" t="s">
         <v>576</v>
       </c>
     </row>
     <row r="232" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A232" s="18" t="s">
+      <c r="A232" s="4" t="s">
         <v>315</v>
       </c>
-      <c r="B232" s="18" t="s">
+      <c r="B232" s="4" t="s">
         <v>577</v>
       </c>
     </row>
     <row r="233" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A233" s="18" t="s">
+      <c r="A233" s="4" t="s">
         <v>318</v>
       </c>
-      <c r="B233" s="18" t="s">
+      <c r="B233" s="4" t="s">
         <v>578</v>
       </c>
     </row>
     <row r="234" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A234" s="18" t="s">
+      <c r="A234" s="4" t="s">
         <v>322</v>
       </c>
-      <c r="B234" s="18" t="s">
+      <c r="B234" s="4" t="s">
         <v>579</v>
       </c>
     </row>
     <row r="235" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A235" s="18" t="s">
+      <c r="A235" s="4" t="s">
         <v>325</v>
       </c>
-      <c r="B235" s="18" t="s">
+      <c r="B235" s="4" t="s">
         <v>580</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="43">
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A27:B28"/>
+    <mergeCell ref="A36:B37"/>
+    <mergeCell ref="A43:B44"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A107:B108"/>
+    <mergeCell ref="A123:B124"/>
+    <mergeCell ref="A133:B134"/>
+    <mergeCell ref="A141:B142"/>
+    <mergeCell ref="A150:B151"/>
+    <mergeCell ref="A125:B125"/>
+    <mergeCell ref="A109:B109"/>
+    <mergeCell ref="A135:B135"/>
+    <mergeCell ref="A164:B165"/>
+    <mergeCell ref="A166:B166"/>
+    <mergeCell ref="A182:B183"/>
+    <mergeCell ref="A184:B184"/>
+    <mergeCell ref="A152:B152"/>
+    <mergeCell ref="A212:B213"/>
+    <mergeCell ref="A214:B214"/>
+    <mergeCell ref="A225:B226"/>
+    <mergeCell ref="A227:B227"/>
+    <mergeCell ref="A143:B143"/>
+    <mergeCell ref="A200:B201"/>
+    <mergeCell ref="A202:B202"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A99:B99"/>
     <mergeCell ref="A83:B83"/>
@@ -7784,26 +7808,6 @@
     <mergeCell ref="A54:B54"/>
     <mergeCell ref="A45:B45"/>
     <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A212:B213"/>
-    <mergeCell ref="A214:B214"/>
-    <mergeCell ref="A225:B226"/>
-    <mergeCell ref="A227:B227"/>
-    <mergeCell ref="A143:B143"/>
-    <mergeCell ref="A135:B135"/>
-    <mergeCell ref="A164:B165"/>
-    <mergeCell ref="A166:B166"/>
-    <mergeCell ref="A182:B183"/>
-    <mergeCell ref="A184:B184"/>
-    <mergeCell ref="A200:B201"/>
-    <mergeCell ref="A202:B202"/>
-    <mergeCell ref="A107:B108"/>
-    <mergeCell ref="A123:B124"/>
-    <mergeCell ref="A133:B134"/>
-    <mergeCell ref="A141:B142"/>
-    <mergeCell ref="A150:B151"/>
-    <mergeCell ref="A152:B152"/>
-    <mergeCell ref="A125:B125"/>
-    <mergeCell ref="A109:B109"/>
     <mergeCell ref="A52:B53"/>
     <mergeCell ref="A63:B64"/>
     <mergeCell ref="A66:B66"/>
@@ -7813,13 +7817,6 @@
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A11:B12"/>
     <mergeCell ref="A19:B20"/>
-    <mergeCell ref="A27:B28"/>
-    <mergeCell ref="A36:B37"/>
-    <mergeCell ref="A43:B44"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A3:B3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -7841,22 +7838,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="25" t="s">
         <v>448</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="25" t="s">
         <v>449</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
@@ -8160,22 +8157,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="27" t="s">
         <v>450</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="27" t="s">
         <v>449</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
@@ -8481,22 +8478,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="27" t="s">
         <v>451</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="27" t="s">
         <v>449</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
@@ -9628,7 +9625,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
docs(BRD): Cập nhật ngôn ngữ Data Warehouse cho Dashboard 1 (Hoạt động tài chính) và chuẩn hóa tên cột
</commit_message>
<xml_diff>
--- a/2. Tài liệu phân tích và thiết kế/04. Mô hình dữ liệu/Data_Dictionary_GML.xlsx
+++ b/2. Tài liệu phân tích và thiết kế/04. Mô hình dữ liệu/Data_Dictionary_GML.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Công việc\1. Dự án Gỗ Minh Long\2. Tài liệu phân tích và thiết kế\04. Mô hình dữ liệu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C2ADBB3-A600-4C16-959F-B1150873A87A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E40781E-8862-4371-A144-62F8103AF662}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11472" yWindow="756" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Danh mục " sheetId="21" r:id="rId1"/>
@@ -1732,9 +1732,6 @@
     <t>Hạn mức vay thực tế được cấp.</t>
   </si>
   <si>
-    <t>Tổng dư nợ gốc hiện tại đang vay.</t>
-  </si>
-  <si>
     <t>Room tín dụng còn lại được phép giải ngân.</t>
   </si>
   <si>
@@ -1921,6 +1918,9 @@
   <si>
     <t>20. fact_collateral (Tài sản Đảm bảo / Thế chấp)</t>
   </si>
+  <si>
+    <t>Dư nợ gốc vay đến hiện tại.</t>
+  </si>
 </sst>
 </file>
 
@@ -1938,6 +1938,7 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -2131,12 +2132,6 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2154,6 +2149,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2471,16 +2472,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05C66EEC-8ED1-44E4-8A82-A486CBBDACC9}">
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="47.28515625" customWidth="1"/>
-    <col min="3" max="3" width="26.42578125" customWidth="1"/>
-    <col min="4" max="4" width="12.28515625" customWidth="1"/>
-    <col min="5" max="5" width="73.7109375" customWidth="1"/>
-    <col min="6" max="6" width="33.5703125" customWidth="1"/>
+    <col min="2" max="2" width="47.33203125" customWidth="1"/>
+    <col min="3" max="3" width="26.44140625" customWidth="1"/>
+    <col min="4" max="4" width="12.33203125" customWidth="1"/>
+    <col min="5" max="5" width="73.6640625" customWidth="1"/>
+    <col min="6" max="6" width="33.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="6" customFormat="1" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -2500,7 +2501,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -2700,7 +2701,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
         <v>11</v>
       </c>
@@ -2760,7 +2761,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <v>14</v>
       </c>
@@ -2908,11 +2909,11 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="18.85546875" customWidth="1"/>
+    <col min="3" max="3" width="18.88671875" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="25" customWidth="1"/>
@@ -3061,7 +3062,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>6</v>
       </c>
@@ -3295,7 +3296,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
@@ -3385,7 +3386,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>3</v>
       </c>
@@ -3406,7 +3407,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>4</v>
       </c>
@@ -3444,7 +3445,7 @@
       </c>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>6</v>
       </c>
@@ -3467,7 +3468,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>7</v>
       </c>
@@ -3490,7 +3491,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>8</v>
       </c>
@@ -3513,7 +3514,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>9</v>
       </c>
@@ -3576,7 +3577,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>12</v>
       </c>
@@ -3614,7 +3615,7 @@
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
     </row>
-    <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>14</v>
       </c>
@@ -3648,7 +3649,7 @@
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
     </row>
-    <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>16</v>
       </c>
@@ -3677,7 +3678,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:G14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
@@ -3769,7 +3770,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>3</v>
       </c>
@@ -3792,7 +3793,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>4</v>
       </c>
@@ -3836,7 +3837,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>6</v>
       </c>
@@ -3874,7 +3875,7 @@
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>8</v>
       </c>
@@ -3908,7 +3909,7 @@
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
     </row>
-    <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>10</v>
       </c>
@@ -3937,7 +3938,7 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -4050,7 +4051,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>4</v>
       </c>
@@ -4071,7 +4072,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>5</v>
       </c>
@@ -4092,7 +4093,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>6</v>
       </c>
@@ -4113,7 +4114,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>7</v>
       </c>
@@ -4136,7 +4137,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>8</v>
       </c>
@@ -4157,7 +4158,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>9</v>
       </c>
@@ -4178,7 +4179,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>10</v>
       </c>
@@ -4199,7 +4200,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>11</v>
       </c>
@@ -4220,7 +4221,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>12</v>
       </c>
@@ -4260,7 +4261,7 @@
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
     </row>
-    <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>14</v>
       </c>
@@ -4294,7 +4295,7 @@
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
     </row>
-    <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>16</v>
       </c>
@@ -4323,7 +4324,7 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
@@ -4413,7 +4414,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>3</v>
       </c>
@@ -4436,7 +4437,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>4</v>
       </c>
@@ -4457,7 +4458,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>5</v>
       </c>
@@ -4478,7 +4479,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>6</v>
       </c>
@@ -4499,7 +4500,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>7</v>
       </c>
@@ -4533,7 +4534,7 @@
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
     </row>
-    <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>9</v>
       </c>
@@ -4562,14 +4563,14 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
     <col min="5" max="5" width="27" customWidth="1"/>
-    <col min="6" max="6" width="39.140625" customWidth="1"/>
+    <col min="6" max="6" width="39.109375" customWidth="1"/>
     <col min="7" max="7" width="17" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4615,7 +4616,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -4659,7 +4660,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -4680,7 +4681,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -4714,7 +4715,7 @@
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
     </row>
-    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -4731,7 +4732,7 @@
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
     </row>
-    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="F11" s="10" t="s">
         <v>437</v>
       </c>
@@ -4749,7 +4750,7 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>
@@ -4839,7 +4840,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>3</v>
       </c>
@@ -4862,7 +4863,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>4</v>
       </c>
@@ -4883,7 +4884,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>5</v>
       </c>
@@ -4904,7 +4905,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>6</v>
       </c>
@@ -4938,7 +4939,7 @@
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>8</v>
       </c>
@@ -4967,7 +4968,7 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:G19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
@@ -5036,7 +5037,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>2</v>
       </c>
@@ -5057,7 +5058,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>3</v>
       </c>
@@ -5122,7 +5123,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>6</v>
       </c>
@@ -5143,7 +5144,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>7</v>
       </c>
@@ -5263,7 +5264,7 @@
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
     </row>
-    <row r="17" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>13</v>
       </c>
@@ -5297,7 +5298,7 @@
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
     </row>
-    <row r="19" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>15</v>
       </c>
@@ -5326,7 +5327,7 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1:G22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
@@ -5355,7 +5356,7 @@
       <c r="D2" s="25"/>
       <c r="E2" s="25"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -5418,7 +5419,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>3</v>
       </c>
@@ -5439,7 +5440,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>4</v>
       </c>
@@ -5481,7 +5482,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>6</v>
       </c>
@@ -5502,7 +5503,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>7</v>
       </c>
@@ -5525,7 +5526,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>8</v>
       </c>
@@ -5546,7 +5547,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>9</v>
       </c>
@@ -5567,7 +5568,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>10</v>
       </c>
@@ -5588,7 +5589,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>11</v>
       </c>
@@ -5609,7 +5610,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>12</v>
       </c>
@@ -5630,7 +5631,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>13</v>
       </c>
@@ -5651,7 +5652,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>14</v>
       </c>
@@ -5689,7 +5690,7 @@
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
     </row>
-    <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>16</v>
       </c>
@@ -5723,7 +5724,7 @@
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
     </row>
-    <row r="22" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>18</v>
       </c>
@@ -5751,11 +5752,11 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <dimension ref="A1:G22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="29" customWidth="1"/>
@@ -5822,7 +5823,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>2</v>
       </c>
@@ -6169,28 +6170,28 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB90C9B3-88E6-4AAB-8063-CEA9E4C03D1B}">
   <dimension ref="A1:B235"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="41.85546875" style="11" customWidth="1"/>
+    <col min="1" max="1" width="41.88671875" style="11" customWidth="1"/>
     <col min="2" max="2" width="41" style="11" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="11"/>
+    <col min="3" max="16384" width="9.109375" style="11"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="21" t="s">
         <v>452</v>
       </c>
-      <c r="B1" s="16"/>
+      <c r="B1" s="22"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="23"/>
       <c r="B2" s="24"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="17" t="s">
-        <v>583</v>
-      </c>
-      <c r="B3" s="18"/>
+      <c r="A3" s="15" t="s">
+        <v>582</v>
+      </c>
+      <c r="B3" s="16"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="13"/>
@@ -6204,7 +6205,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>13</v>
       </c>
@@ -6212,7 +6213,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>18</v>
       </c>
@@ -6236,27 +6237,27 @@
         <v>458</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>30</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="17"/>
+      <c r="B11" s="18"/>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="19"/>
+      <c r="B12" s="20"/>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="15" t="s">
         <v>584</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="19"/>
-      <c r="B11" s="20"/>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="21"/>
-      <c r="B12" s="22"/>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="17" t="s">
-        <v>585</v>
-      </c>
-      <c r="B13" s="18"/>
+      <c r="B13" s="16"/>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="13"/>
@@ -6270,7 +6271,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>44</v>
       </c>
@@ -6278,7 +6279,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>47</v>
       </c>
@@ -6286,7 +6287,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>50</v>
       </c>
@@ -6295,18 +6296,18 @@
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="19"/>
-      <c r="B19" s="20"/>
+      <c r="A19" s="17"/>
+      <c r="B19" s="18"/>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="21"/>
-      <c r="B20" s="22"/>
+      <c r="A20" s="19"/>
+      <c r="B20" s="20"/>
     </row>
     <row r="21" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="17" t="s">
-        <v>586</v>
-      </c>
-      <c r="B21" s="18"/>
+      <c r="A21" s="15" t="s">
+        <v>585</v>
+      </c>
+      <c r="B21" s="16"/>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="13"/>
@@ -6320,7 +6321,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
         <v>53</v>
       </c>
@@ -6345,18 +6346,18 @@
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="19"/>
-      <c r="B27" s="20"/>
+      <c r="A27" s="17"/>
+      <c r="B27" s="18"/>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="21"/>
-      <c r="B28" s="22"/>
+      <c r="A28" s="19"/>
+      <c r="B28" s="20"/>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="17" t="s">
-        <v>587</v>
-      </c>
-      <c r="B29" s="18"/>
+      <c r="A29" s="15" t="s">
+        <v>586</v>
+      </c>
+      <c r="B29" s="16"/>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="13"/>
@@ -6370,7 +6371,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
         <v>60</v>
       </c>
@@ -6386,7 +6387,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
         <v>66</v>
       </c>
@@ -6403,18 +6404,18 @@
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" s="19"/>
-      <c r="B36" s="20"/>
+      <c r="A36" s="17"/>
+      <c r="B36" s="18"/>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" s="21"/>
-      <c r="B37" s="22"/>
+      <c r="A37" s="19"/>
+      <c r="B37" s="20"/>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" s="17" t="s">
-        <v>588</v>
-      </c>
-      <c r="B38" s="18"/>
+      <c r="A38" s="15" t="s">
+        <v>587</v>
+      </c>
+      <c r="B38" s="16"/>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="13"/>
@@ -6428,7 +6429,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
         <v>69</v>
       </c>
@@ -6445,18 +6446,18 @@
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="19"/>
-      <c r="B43" s="20"/>
+      <c r="A43" s="17"/>
+      <c r="B43" s="18"/>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" s="21"/>
-      <c r="B44" s="22"/>
+      <c r="A44" s="19"/>
+      <c r="B44" s="20"/>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" s="17" t="s">
-        <v>589</v>
-      </c>
-      <c r="B45" s="18"/>
+      <c r="A45" s="15" t="s">
+        <v>588</v>
+      </c>
+      <c r="B45" s="16"/>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="13"/>
@@ -6478,7 +6479,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="49" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
         <v>78</v>
       </c>
@@ -6494,7 +6495,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
         <v>84</v>
       </c>
@@ -6503,18 +6504,18 @@
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A52" s="19"/>
-      <c r="B52" s="20"/>
+      <c r="A52" s="17"/>
+      <c r="B52" s="18"/>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A53" s="21"/>
-      <c r="B53" s="22"/>
+      <c r="A53" s="19"/>
+      <c r="B53" s="20"/>
     </row>
     <row r="54" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="17" t="s">
-        <v>590</v>
-      </c>
-      <c r="B54" s="18"/>
+      <c r="A54" s="15" t="s">
+        <v>589</v>
+      </c>
+      <c r="B54" s="16"/>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="13"/>
@@ -6528,7 +6529,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="57" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
         <v>87</v>
       </c>
@@ -6536,15 +6537,15 @@
         <v>475</v>
       </c>
     </row>
-    <row r="58" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
         <v>89</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>591</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
         <v>92</v>
       </c>
@@ -6560,7 +6561,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="61" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="s">
         <v>97</v>
       </c>
@@ -6568,7 +6569,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="62" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
         <v>100</v>
       </c>
@@ -6577,28 +6578,28 @@
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A63" s="19"/>
-      <c r="B63" s="20"/>
+      <c r="A63" s="17"/>
+      <c r="B63" s="18"/>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A64" s="21"/>
-      <c r="B64" s="22"/>
+      <c r="A64" s="19"/>
+      <c r="B64" s="20"/>
     </row>
     <row r="65" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="15" t="s">
+      <c r="A65" s="21" t="s">
         <v>480</v>
       </c>
-      <c r="B65" s="16"/>
+      <c r="B65" s="22"/>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="23"/>
       <c r="B66" s="24"/>
     </row>
     <row r="67" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="17" t="s">
-        <v>592</v>
-      </c>
-      <c r="B67" s="18"/>
+      <c r="A67" s="15" t="s">
+        <v>591</v>
+      </c>
+      <c r="B67" s="16"/>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" s="13"/>
@@ -6628,7 +6629,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="72" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
         <v>111</v>
       </c>
@@ -6701,18 +6702,18 @@
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A81" s="19"/>
-      <c r="B81" s="20"/>
+      <c r="A81" s="17"/>
+      <c r="B81" s="18"/>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A82" s="21"/>
-      <c r="B82" s="22"/>
+      <c r="A82" s="19"/>
+      <c r="B82" s="20"/>
     </row>
     <row r="83" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="17" t="s">
-        <v>593</v>
-      </c>
-      <c r="B83" s="18"/>
+      <c r="A83" s="15" t="s">
+        <v>592</v>
+      </c>
+      <c r="B83" s="16"/>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" s="13"/>
@@ -6815,18 +6816,18 @@
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A97" s="19"/>
-      <c r="B97" s="20"/>
+      <c r="A97" s="17"/>
+      <c r="B97" s="18"/>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A98" s="21"/>
-      <c r="B98" s="22"/>
+      <c r="A98" s="19"/>
+      <c r="B98" s="20"/>
     </row>
     <row r="99" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A99" s="17" t="s">
-        <v>594</v>
-      </c>
-      <c r="B99" s="18"/>
+      <c r="A99" s="15" t="s">
+        <v>593</v>
+      </c>
+      <c r="B99" s="16"/>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" s="13"/>
@@ -6881,18 +6882,18 @@
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A107" s="19"/>
-      <c r="B107" s="20"/>
+      <c r="A107" s="17"/>
+      <c r="B107" s="18"/>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A108" s="21"/>
-      <c r="B108" s="22"/>
+      <c r="A108" s="19"/>
+      <c r="B108" s="20"/>
     </row>
     <row r="109" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="17" t="s">
-        <v>595</v>
-      </c>
-      <c r="B109" s="18"/>
+      <c r="A109" s="15" t="s">
+        <v>594</v>
+      </c>
+      <c r="B109" s="16"/>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110" s="13"/>
@@ -6922,7 +6923,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="114" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A114" s="4" t="s">
         <v>108</v>
       </c>
@@ -6946,7 +6947,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="117" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A117" s="4" t="s">
         <v>13</v>
       </c>
@@ -6954,12 +6955,12 @@
         <v>513</v>
       </c>
     </row>
-    <row r="118" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A118" s="4" t="s">
         <v>177</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.25">
@@ -6967,7 +6968,7 @@
         <v>179</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.25">
@@ -6995,18 +6996,18 @@
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A123" s="19"/>
-      <c r="B123" s="20"/>
+      <c r="A123" s="17"/>
+      <c r="B123" s="18"/>
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A124" s="21"/>
-      <c r="B124" s="22"/>
+      <c r="A124" s="19"/>
+      <c r="B124" s="20"/>
     </row>
     <row r="125" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A125" s="17" t="s">
-        <v>596</v>
-      </c>
-      <c r="B125" s="18"/>
+      <c r="A125" s="15" t="s">
+        <v>595</v>
+      </c>
+      <c r="B125" s="16"/>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A126" s="13"/>
@@ -7061,18 +7062,18 @@
       </c>
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A133" s="19"/>
-      <c r="B133" s="20"/>
+      <c r="A133" s="17"/>
+      <c r="B133" s="18"/>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A134" s="21"/>
-      <c r="B134" s="22"/>
+      <c r="A134" s="19"/>
+      <c r="B134" s="20"/>
     </row>
     <row r="135" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A135" s="17" t="s">
-        <v>597</v>
-      </c>
-      <c r="B135" s="18"/>
+      <c r="A135" s="15" t="s">
+        <v>596</v>
+      </c>
+      <c r="B135" s="16"/>
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A136" s="13"/>
@@ -7086,7 +7087,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="138" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A138" s="4" t="s">
         <v>190</v>
       </c>
@@ -7111,18 +7112,18 @@
       </c>
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A141" s="19"/>
-      <c r="B141" s="20"/>
+      <c r="A141" s="17"/>
+      <c r="B141" s="18"/>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A142" s="21"/>
-      <c r="B142" s="22"/>
+      <c r="A142" s="19"/>
+      <c r="B142" s="20"/>
     </row>
     <row r="143" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A143" s="17" t="s">
-        <v>598</v>
-      </c>
-      <c r="B143" s="18"/>
+      <c r="A143" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="B143" s="16"/>
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A144" s="13"/>
@@ -7169,18 +7170,18 @@
       </c>
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A150" s="19"/>
-      <c r="B150" s="20"/>
+      <c r="A150" s="17"/>
+      <c r="B150" s="18"/>
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A151" s="21"/>
-      <c r="B151" s="22"/>
+      <c r="A151" s="19"/>
+      <c r="B151" s="20"/>
     </row>
     <row r="152" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A152" s="17" t="s">
-        <v>599</v>
-      </c>
-      <c r="B152" s="18"/>
+      <c r="A152" s="15" t="s">
+        <v>598</v>
+      </c>
+      <c r="B152" s="16"/>
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A153" s="13"/>
@@ -7267,18 +7268,18 @@
       </c>
     </row>
     <row r="164" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A164" s="19"/>
-      <c r="B164" s="20"/>
+      <c r="A164" s="17"/>
+      <c r="B164" s="18"/>
     </row>
     <row r="165" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A165" s="21"/>
-      <c r="B165" s="22"/>
+      <c r="A165" s="19"/>
+      <c r="B165" s="20"/>
     </row>
     <row r="166" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A166" s="17" t="s">
-        <v>600</v>
-      </c>
-      <c r="B166" s="18"/>
+      <c r="A166" s="15" t="s">
+        <v>599</v>
+      </c>
+      <c r="B166" s="16"/>
     </row>
     <row r="167" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A167" s="13"/>
@@ -7356,7 +7357,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="177" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A177" s="4" t="s">
         <v>179</v>
       </c>
@@ -7364,7 +7365,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="178" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A178" s="4" t="s">
         <v>261</v>
       </c>
@@ -7372,7 +7373,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="179" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A179" s="4" t="s">
         <v>264</v>
       </c>
@@ -7397,18 +7398,18 @@
       </c>
     </row>
     <row r="182" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A182" s="19"/>
-      <c r="B182" s="20"/>
+      <c r="A182" s="17"/>
+      <c r="B182" s="18"/>
     </row>
     <row r="183" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A183" s="21"/>
-      <c r="B183" s="22"/>
+      <c r="A183" s="19"/>
+      <c r="B183" s="20"/>
     </row>
     <row r="184" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A184" s="17" t="s">
-        <v>601</v>
-      </c>
-      <c r="B184" s="18"/>
+      <c r="A184" s="15" t="s">
+        <v>600</v>
+      </c>
+      <c r="B184" s="16"/>
     </row>
     <row r="185" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A185" s="13"/>
@@ -7422,7 +7423,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="187" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A187" s="4" t="s">
         <v>104</v>
       </c>
@@ -7478,7 +7479,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="194" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A194" s="4" t="s">
         <v>177</v>
       </c>
@@ -7486,7 +7487,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="195" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A195" s="4" t="s">
         <v>179</v>
       </c>
@@ -7494,7 +7495,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="196" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A196" s="4" t="s">
         <v>264</v>
       </c>
@@ -7502,7 +7503,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="197" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A197" s="4" t="s">
         <v>261</v>
       </c>
@@ -7527,18 +7528,18 @@
       </c>
     </row>
     <row r="200" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A200" s="19"/>
-      <c r="B200" s="20"/>
+      <c r="A200" s="17"/>
+      <c r="B200" s="18"/>
     </row>
     <row r="201" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A201" s="21"/>
-      <c r="B201" s="22"/>
+      <c r="A201" s="19"/>
+      <c r="B201" s="20"/>
     </row>
     <row r="202" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A202" s="17" t="s">
-        <v>602</v>
-      </c>
-      <c r="B202" s="18"/>
+      <c r="A202" s="15" t="s">
+        <v>601</v>
+      </c>
+      <c r="B202" s="16"/>
     </row>
     <row r="203" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A203" s="13"/>
@@ -7560,7 +7561,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="206" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A206" s="4" t="s">
         <v>276</v>
       </c>
@@ -7581,7 +7582,7 @@
         <v>279</v>
       </c>
       <c r="B208" s="4" t="s">
-        <v>563</v>
+        <v>604</v>
       </c>
     </row>
     <row r="209" spans="1:2" x14ac:dyDescent="0.25">
@@ -7589,7 +7590,7 @@
         <v>282</v>
       </c>
       <c r="B209" s="4" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="210" spans="1:2" x14ac:dyDescent="0.25">
@@ -7597,7 +7598,7 @@
         <v>286</v>
       </c>
       <c r="B210" s="4" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="211" spans="1:2" x14ac:dyDescent="0.25">
@@ -7605,22 +7606,22 @@
         <v>227</v>
       </c>
       <c r="B211" s="4" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="212" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A212" s="19"/>
-      <c r="B212" s="20"/>
+      <c r="A212" s="17"/>
+      <c r="B212" s="18"/>
     </row>
     <row r="213" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A213" s="21"/>
-      <c r="B213" s="22"/>
+      <c r="A213" s="19"/>
+      <c r="B213" s="20"/>
     </row>
     <row r="214" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A214" s="17" t="s">
-        <v>603</v>
-      </c>
-      <c r="B214" s="18"/>
+      <c r="A214" s="15" t="s">
+        <v>602</v>
+      </c>
+      <c r="B214" s="16"/>
     </row>
     <row r="215" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A215" s="13"/>
@@ -7639,15 +7640,15 @@
         <v>304</v>
       </c>
       <c r="B217" s="4" t="s">
-        <v>567</v>
-      </c>
-    </row>
-    <row r="218" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A218" s="4" t="s">
         <v>242</v>
       </c>
       <c r="B218" s="4" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="219" spans="1:2" x14ac:dyDescent="0.25">
@@ -7655,7 +7656,7 @@
         <v>60</v>
       </c>
       <c r="B219" s="4" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="220" spans="1:2" x14ac:dyDescent="0.25">
@@ -7663,7 +7664,7 @@
         <v>293</v>
       </c>
       <c r="B220" s="4" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="221" spans="1:2" x14ac:dyDescent="0.25">
@@ -7671,7 +7672,7 @@
         <v>296</v>
       </c>
       <c r="B221" s="4" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
     <row r="222" spans="1:2" x14ac:dyDescent="0.25">
@@ -7679,7 +7680,7 @@
         <v>299</v>
       </c>
       <c r="B222" s="4" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
     </row>
     <row r="223" spans="1:2" x14ac:dyDescent="0.25">
@@ -7687,30 +7688,30 @@
         <v>308</v>
       </c>
       <c r="B223" s="4" t="s">
-        <v>573</v>
-      </c>
-    </row>
-    <row r="224" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A224" s="4" t="s">
         <v>227</v>
       </c>
       <c r="B224" s="4" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="225" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A225" s="19"/>
-      <c r="B225" s="20"/>
+      <c r="A225" s="17"/>
+      <c r="B225" s="18"/>
     </row>
     <row r="226" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A226" s="21"/>
-      <c r="B226" s="22"/>
+      <c r="A226" s="19"/>
+      <c r="B226" s="20"/>
     </row>
     <row r="227" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A227" s="17" t="s">
-        <v>604</v>
-      </c>
-      <c r="B227" s="18"/>
+      <c r="A227" s="15" t="s">
+        <v>603</v>
+      </c>
+      <c r="B227" s="16"/>
     </row>
     <row r="228" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A228" s="13"/>
@@ -7729,15 +7730,15 @@
         <v>60</v>
       </c>
       <c r="B230" s="4" t="s">
-        <v>575</v>
-      </c>
-    </row>
-    <row r="231" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A231" s="4" t="s">
         <v>312</v>
       </c>
       <c r="B231" s="4" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
     <row r="232" spans="1:2" x14ac:dyDescent="0.25">
@@ -7745,15 +7746,15 @@
         <v>315</v>
       </c>
       <c r="B232" s="4" t="s">
-        <v>577</v>
-      </c>
-    </row>
-    <row r="233" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="233" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A233" s="4" t="s">
         <v>318</v>
       </c>
       <c r="B233" s="4" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="234" spans="1:2" x14ac:dyDescent="0.25">
@@ -7761,46 +7762,19 @@
         <v>322</v>
       </c>
       <c r="B234" s="4" t="s">
-        <v>579</v>
-      </c>
-    </row>
-    <row r="235" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="235" spans="1:2" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A235" s="4" t="s">
         <v>325</v>
       </c>
       <c r="B235" s="4" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="43">
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A27:B28"/>
-    <mergeCell ref="A36:B37"/>
-    <mergeCell ref="A43:B44"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A107:B108"/>
-    <mergeCell ref="A123:B124"/>
-    <mergeCell ref="A133:B134"/>
-    <mergeCell ref="A141:B142"/>
-    <mergeCell ref="A150:B151"/>
-    <mergeCell ref="A125:B125"/>
-    <mergeCell ref="A109:B109"/>
-    <mergeCell ref="A135:B135"/>
-    <mergeCell ref="A164:B165"/>
-    <mergeCell ref="A166:B166"/>
-    <mergeCell ref="A182:B183"/>
-    <mergeCell ref="A184:B184"/>
-    <mergeCell ref="A152:B152"/>
-    <mergeCell ref="A212:B213"/>
-    <mergeCell ref="A214:B214"/>
-    <mergeCell ref="A225:B226"/>
-    <mergeCell ref="A227:B227"/>
-    <mergeCell ref="A143:B143"/>
-    <mergeCell ref="A200:B201"/>
-    <mergeCell ref="A202:B202"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A99:B99"/>
     <mergeCell ref="A83:B83"/>
@@ -7817,6 +7791,33 @@
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A11:B12"/>
     <mergeCell ref="A19:B20"/>
+    <mergeCell ref="A212:B213"/>
+    <mergeCell ref="A214:B214"/>
+    <mergeCell ref="A225:B226"/>
+    <mergeCell ref="A227:B227"/>
+    <mergeCell ref="A143:B143"/>
+    <mergeCell ref="A200:B201"/>
+    <mergeCell ref="A202:B202"/>
+    <mergeCell ref="A164:B165"/>
+    <mergeCell ref="A166:B166"/>
+    <mergeCell ref="A182:B183"/>
+    <mergeCell ref="A184:B184"/>
+    <mergeCell ref="A152:B152"/>
+    <mergeCell ref="A107:B108"/>
+    <mergeCell ref="A123:B124"/>
+    <mergeCell ref="A133:B134"/>
+    <mergeCell ref="A141:B142"/>
+    <mergeCell ref="A150:B151"/>
+    <mergeCell ref="A125:B125"/>
+    <mergeCell ref="A109:B109"/>
+    <mergeCell ref="A135:B135"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A27:B28"/>
+    <mergeCell ref="A36:B37"/>
+    <mergeCell ref="A43:B44"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A21:B21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -7826,7 +7827,7 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
@@ -7897,7 +7898,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>2</v>
       </c>
@@ -7920,7 +7921,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>3</v>
       </c>
@@ -7941,7 +7942,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>4</v>
       </c>
@@ -7962,7 +7963,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>5</v>
       </c>
@@ -7983,7 +7984,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>6</v>
       </c>
@@ -8004,7 +8005,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>7</v>
       </c>
@@ -8046,7 +8047,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>9</v>
       </c>
@@ -8082,7 +8083,7 @@
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
     </row>
-    <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>11</v>
       </c>
@@ -8116,7 +8117,7 @@
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
     </row>
-    <row r="17" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>13</v>
       </c>
@@ -8145,7 +8146,7 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
   <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
@@ -8216,7 +8217,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>2</v>
       </c>
@@ -8239,7 +8240,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>3</v>
       </c>
@@ -8260,7 +8261,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>4</v>
       </c>
@@ -8281,7 +8282,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>5</v>
       </c>
@@ -8365,7 +8366,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>9</v>
       </c>
@@ -8403,7 +8404,7 @@
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
     </row>
-    <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>11</v>
       </c>
@@ -8437,7 +8438,7 @@
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
     </row>
-    <row r="17" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>13</v>
       </c>
@@ -8466,12 +8467,12 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
   <dimension ref="A1:G15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.44140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="37" customWidth="1"/>
     <col min="7" max="7" width="24" customWidth="1"/>
@@ -8747,11 +8748,11 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="16.5703125" customWidth="1"/>
+    <col min="3" max="3" width="16.5546875" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="6" max="6" width="36" customWidth="1"/>
@@ -8979,7 +8980,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="55.2" x14ac:dyDescent="0.25">
       <c r="F13" s="8" t="s">
         <v>418</v>
       </c>
@@ -8992,11 +8993,11 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="18.5703125" customWidth="1"/>
+    <col min="3" max="3" width="18.5546875" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="6" max="6" width="48" customWidth="1"/>
@@ -9179,7 +9180,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -9276,7 +9277,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -9368,7 +9369,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -9421,7 +9422,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -9572,10 +9573,10 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="18.140625" customWidth="1"/>
+    <col min="2" max="2" width="18.109375" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
@@ -9648,7 +9649,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -9738,11 +9739,11 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="18.42578125" customWidth="1"/>
+    <col min="3" max="3" width="18.44140625" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="6" max="6" width="40" customWidth="1"/>
@@ -9814,7 +9815,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -9946,11 +9947,11 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:G15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" customWidth="1"/>
+    <col min="3" max="3" width="19.6640625" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="6" max="6" width="43" customWidth="1"/>

</xml_diff>